<commit_message>
Update WS1_Complete_Solution and BOM with revised desktop versions
</commit_message>
<xml_diff>
--- a/WS1_Power_BOM_Completed.xlsx
+++ b/WS1_Power_BOM_Completed.xlsx
@@ -551,7 +551,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>505-1973-1-ND</t>
+          <t>505-LTC3112EFE#PBF-ND</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>I2C. Needs 1.8V VDD + 3.3V VLED</t>
+          <t>SpO2 + HR, I2C</t>
         </is>
       </c>
     </row>
@@ -1202,7 +1202,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>8-60s non-volatile recording</t>
+          <t>8-60s non-volatile recording. DigiKey does not stock bare IC; available via Grove module or AliExpress</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>AOM-4544P-2-R</t>
+          <t>CMA-4544PF-W</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Omni-directional. For APR9600 audio input</t>
+          <t>Omni-directional. For APR9600 audio input. Verified DigiKey stock: 12,444</t>
         </is>
       </c>
     </row>
@@ -1643,22 +1643,22 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>668-1628-ND</t>
+          <t>GF0668-ND</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>PSR-28N08A-JQ</t>
+          <t>GF0668</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>28mm</t>
+          <t>66x66mm</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>4Ω, 3W. Drives by PAM8406 Class D amp</t>
+          <t>8Ω, 3W. DigiKey verified stock: 8,654. Drives by PAM8406 Class D amp</t>
         </is>
       </c>
     </row>

</xml_diff>